<commit_message>
Aquisição 100% outbound por ligação: sem anúncios, Places API, 0303; planilha atualizada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuMCmqDPYgwMtrBRrEVBkM
</commit_message>
<xml_diff>
--- a/empresa/financeiro/custos-recepcao-ia.xlsx
+++ b/empresa/financeiro/custos-recepcao-ia.xlsx
@@ -529,19 +529,19 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>107</v>
@@ -760,27 +760,27 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>-'Custos mensais'!D17</f>
+        <f>-'Custos mensais'!D18</f>
         <v/>
       </c>
       <c r="C9" s="3">
-        <f>-'Custos mensais'!E17</f>
+        <f>-'Custos mensais'!E18</f>
         <v/>
       </c>
       <c r="D9" s="3">
-        <f>-'Custos mensais'!F17</f>
+        <f>-'Custos mensais'!F18</f>
         <v/>
       </c>
       <c r="E9" s="3">
-        <f>-'Custos mensais'!G17</f>
+        <f>-'Custos mensais'!G18</f>
         <v/>
       </c>
       <c r="F9" s="3">
-        <f>-'Custos mensais'!H17</f>
+        <f>-'Custos mensais'!H18</f>
         <v/>
       </c>
       <c r="G9" s="3">
-        <f>-'Custos mensais'!I17</f>
+        <f>-'Custos mensais'!I18</f>
         <v/>
       </c>
       <c r="H9" s="3">
@@ -795,27 +795,27 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>-'Custos mensais'!D18</f>
+        <f>-'Custos mensais'!D19</f>
         <v/>
       </c>
       <c r="C10" s="3">
-        <f>-'Custos mensais'!E18</f>
+        <f>-'Custos mensais'!E19</f>
         <v/>
       </c>
       <c r="D10" s="3">
-        <f>-'Custos mensais'!F18</f>
+        <f>-'Custos mensais'!F19</f>
         <v/>
       </c>
       <c r="E10" s="3">
-        <f>-'Custos mensais'!G18</f>
+        <f>-'Custos mensais'!G19</f>
         <v/>
       </c>
       <c r="F10" s="3">
-        <f>-'Custos mensais'!H18</f>
+        <f>-'Custos mensais'!H19</f>
         <v/>
       </c>
       <c r="G10" s="3">
-        <f>-'Custos mensais'!I18</f>
+        <f>-'Custos mensais'!I19</f>
         <v/>
       </c>
       <c r="H10" s="3">
@@ -998,31 +998,31 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAC (mídia + ligações ÷ clientes novos)</t>
+          <t>CAC (ligações ÷ clientes novos)</t>
         </is>
       </c>
       <c r="B16" s="3">
-        <f>IF(B3&gt;0,(-B10+'Custos mensais'!D15)/B3,0)</f>
+        <f>IF(B3&gt;0,(-B10+'Custos mensais'!D16)/B3,0)</f>
         <v/>
       </c>
       <c r="C16" s="3">
-        <f>IF(C3&gt;0,(-C10+'Custos mensais'!E15)/C3,0)</f>
+        <f>IF(C3&gt;0,(-C10+'Custos mensais'!E16)/C3,0)</f>
         <v/>
       </c>
       <c r="D16" s="3">
-        <f>IF(D3&gt;0,(-D10+'Custos mensais'!F15)/D3,0)</f>
+        <f>IF(D3&gt;0,(-D10+'Custos mensais'!F16)/D3,0)</f>
         <v/>
       </c>
       <c r="E16" s="3">
-        <f>IF(E3&gt;0,(-E10+'Custos mensais'!G15)/E3,0)</f>
+        <f>IF(E3&gt;0,(-E10+'Custos mensais'!G16)/E3,0)</f>
         <v/>
       </c>
       <c r="F16" s="3">
-        <f>IF(F3&gt;0,(-F10+'Custos mensais'!H15)/F3,0)</f>
+        <f>IF(F3&gt;0,(-F10+'Custos mensais'!H16)/F3,0)</f>
         <v/>
       </c>
       <c r="G16" s="3">
-        <f>IF(G3&gt;0,(-G10+'Custos mensais'!I15)/G3,0)</f>
+        <f>IF(G3&gt;0,(-G10+'Custos mensais'!I16)/G3,0)</f>
         <v/>
       </c>
     </row>
@@ -1210,13 +1210,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Minutos por ligação</t>
+          <t>Minutos médios por ligação</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
+        <v>1.5</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mistura de não atendidas (~0,5 min) e conversas (3–5 min)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1229,7 +1233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1407,22 +1411,22 @@
         </is>
       </c>
       <c r="D4" s="12" t="n">
-        <v>22</v>
+        <v>99</v>
       </c>
       <c r="E4" s="12" t="n">
-        <v>22</v>
+        <v>99</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>99</v>
+        <v>330</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>99</v>
+        <v>330</v>
       </c>
       <c r="H4" s="12" t="n">
-        <v>99</v>
+        <v>330</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>99</v>
+        <v>330</v>
       </c>
       <c r="J4" s="3">
         <f>IF(C4="R$",SUM(D4:I4),"")</f>
@@ -1430,7 +1434,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Pro no mês 3 para mais minutos/vozes</t>
+          <t>Pro desde o mês 1; Scale no mês 3 para o volume de ligações</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1530,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Número BR para ligações (Twilio/SIP)</t>
+          <t>Número BR com prefixo 0303 (telemarketing ativo)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1535,22 +1539,22 @@
         </is>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="J7" s="3">
         <f>IF(C7="R$",SUM(D7:I7),"")</f>
@@ -1558,43 +1562,43 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>A partir da Fase 2</t>
+          <t>Exigência Anatel para ligação ativa de oferta</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Telefonia</t>
+          <t>Prospecção</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ligações de venda (nº de ligações)</t>
+          <t>Google Places API (busca de clínicas)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>lig.</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="12" t="n">
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="G8" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="F8" s="12" t="n">
-        <v>300</v>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>500</v>
-      </c>
-      <c r="H8" s="12" t="n">
-        <v>600</v>
-      </c>
-      <c r="I8" s="12" t="n">
-        <v>600</v>
+      <c r="H8" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>100</v>
       </c>
       <c r="J8" s="3">
         <f>IF(C8="R$",SUM(D8:I8),"")</f>
@@ -1602,43 +1606,43 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Edite o volume; custo calculado abaixo</t>
+          <t>Lista por cidade com nota e nº de avaliações</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mídia</t>
+          <t>Telefonia</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>Ligações de venda (nº de ligações)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>R$</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="n">
+          <t>lig.</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>600</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F9" s="12" t="n">
         <v>1500</v>
       </c>
-      <c r="E9" s="11" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>6000</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>8000</v>
-      </c>
-      <c r="I9" s="11" t="n">
-        <v>9000</v>
+      <c r="G9" s="12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H9" s="12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I9" s="12" t="n">
+        <v>2000</v>
       </c>
       <c r="J9" s="3">
         <f>IF(C9="R$",SUM(D9:I9),"")</f>
@@ -1646,19 +1650,19 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Principal alavanca; só sobe com CAC na meta</t>
+          <t>~57 ligações por venda (25% atende decisor × 20% avança × 35% fecha)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Administrativo</t>
+          <t>Mídia</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Contador (após CNPJ)</t>
+          <t>Meta Ads</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1673,16 +1677,16 @@
         <v>0</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="G10" s="11" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H10" s="11" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J10" s="3">
         <f>IF(C10="R$",SUM(D10:I10),"")</f>
@@ -1690,7 +1694,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>CNPJ previsto no fim do mês 2</t>
+          <t>Sem anúncios: aquisição 100% por prospecção ativa</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1706,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Abertura do CNPJ (único)</t>
+          <t>Contador (após CNPJ)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1717,16 +1721,16 @@
         <v>0</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H11" s="11" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="J11" s="3">
         <f>IF(C11="R$",SUM(D11:I11),"")</f>
@@ -1734,19 +1738,19 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Estimativa</t>
+          <t>CNPJ previsto no fim do mês 2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Reserva</t>
+          <t>Administrativo</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Imprevistos (10% dos custos fixos acima)</t>
+          <t>Abertura do CNPJ (único)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1754,29 +1758,23 @@
           <t>R$</t>
         </is>
       </c>
-      <c r="D12" s="3">
-        <f>0.1*(D2+D5+D6+D7+D10+D11+SUM(D13:D15))</f>
-        <v/>
-      </c>
-      <c r="E12" s="3">
-        <f>0.1*(E2+E5+E6+E7+E10+E11+SUM(E13:E15))</f>
-        <v/>
-      </c>
-      <c r="F12" s="3">
-        <f>0.1*(F2+F5+F6+F7+F10+F11+SUM(F13:F15))</f>
-        <v/>
-      </c>
-      <c r="G12" s="3">
-        <f>0.1*(G2+G5+G6+G7+G10+G11+SUM(G13:G15))</f>
-        <v/>
-      </c>
-      <c r="H12" s="3">
-        <f>0.1*(H2+H5+H6+H7+H10+H11+SUM(H13:H15))</f>
-        <v/>
-      </c>
-      <c r="I12" s="3">
-        <f>0.1*(I2+I5+I6+I7+I10+I11+SUM(I13:I15))</f>
-        <v/>
+      <c r="D12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="J12" s="3">
         <f>IF(C12="R$",SUM(D12:I12),"")</f>
@@ -1784,19 +1782,19 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Calculado</t>
+          <t>Estimativa</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Conversões</t>
+          <t>Reserva</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Claude (R$)</t>
+          <t>Imprevistos (10% dos custos fixos acima)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1805,33 +1803,38 @@
         </is>
       </c>
       <c r="D13" s="3">
-        <f>D3*Premissas!$B$2</f>
+        <f>0.1*(D2+D5+D6+D7+D8+D11+D12+SUM(D14:D16))</f>
         <v/>
       </c>
       <c r="E13" s="3">
-        <f>E3*Premissas!$B$2</f>
+        <f>0.1*(E2+E5+E6+E7+E8+E11+E12+SUM(E14:E16))</f>
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>F3*Premissas!$B$2</f>
+        <f>0.1*(F2+F5+F6+F7+F8+F11+F12+SUM(F14:F16))</f>
         <v/>
       </c>
       <c r="G13" s="3">
-        <f>G3*Premissas!$B$2</f>
+        <f>0.1*(G2+G5+G6+G7+G8+G11+G12+SUM(G14:G16))</f>
         <v/>
       </c>
       <c r="H13" s="3">
-        <f>H3*Premissas!$B$2</f>
+        <f>0.1*(H2+H5+H6+H7+H8+H11+H12+SUM(H14:H16))</f>
         <v/>
       </c>
       <c r="I13" s="3">
-        <f>I3*Premissas!$B$2</f>
+        <f>0.1*(I2+I5+I6+I7+I8+I11+I12+SUM(I14:I16))</f>
         <v/>
       </c>
       <c r="J13" s="3">
         <f>IF(C13="R$",SUM(D13:I13),"")</f>
         <v/>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Calculado</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1841,7 +1844,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ElevenLabs (R$)</t>
+          <t>Claude (R$)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1850,27 +1853,27 @@
         </is>
       </c>
       <c r="D14" s="3">
-        <f>D4*Premissas!$B$2</f>
+        <f>D3*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="E14" s="3">
-        <f>E4*Premissas!$B$2</f>
+        <f>E3*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="F14" s="3">
-        <f>F4*Premissas!$B$2</f>
+        <f>F3*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="G14" s="3">
-        <f>G4*Premissas!$B$2</f>
+        <f>G3*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="H14" s="3">
-        <f>H4*Premissas!$B$2</f>
+        <f>H3*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="I14" s="3">
-        <f>I4*Premissas!$B$2</f>
+        <f>I3*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="J14" s="3">
@@ -1886,7 +1889,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Custo das ligações (R$)</t>
+          <t>ElevenLabs (R$)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1895,27 +1898,27 @@
         </is>
       </c>
       <c r="D15" s="3">
-        <f>D8*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <f>D4*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="E15" s="3">
-        <f>E8*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <f>E4*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="F15" s="3">
-        <f>F8*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <f>F4*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="G15" s="3">
-        <f>G8*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <f>G4*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="H15" s="3">
-        <f>H8*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <f>H4*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="I15" s="3">
-        <f>I8*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <f>I4*Premissas!$B$2</f>
         <v/>
       </c>
       <c r="J15" s="3">
@@ -1924,80 +1927,90 @@
       </c>
     </row>
     <row r="16">
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Conversões</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Custo das ligações (R$)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D16" s="3">
+        <f>D9*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <v/>
+      </c>
+      <c r="E16" s="3">
+        <f>E9*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <v/>
+      </c>
+      <c r="F16" s="3">
+        <f>F9*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <v/>
+      </c>
+      <c r="G16" s="3">
+        <f>G9*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <v/>
+      </c>
+      <c r="H16" s="3">
+        <f>H9*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <v/>
+      </c>
+      <c r="I16" s="3">
+        <f>I9*Premissas!$B$10*Premissas!$B$9*Premissas!$B$2</f>
+        <v/>
+      </c>
       <c r="J16" s="3">
         <f>IF(C16="R$",SUM(D16:I16),"")</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>CUSTO OPERACIONAL (sem mídia)</t>
-        </is>
-      </c>
-      <c r="D17" s="5">
-        <f>D2+D5+D6+D7+D10+D11+D12+SUM(D13:D15)</f>
-        <v/>
-      </c>
-      <c r="E17" s="5">
-        <f>E2+E5+E6+E7+E10+E11+E12+SUM(E13:E15)</f>
-        <v/>
-      </c>
-      <c r="F17" s="5">
-        <f>F2+F5+F6+F7+F10+F11+F12+SUM(F13:F15)</f>
-        <v/>
-      </c>
-      <c r="G17" s="5">
-        <f>G2+G5+G6+G7+G10+G11+G12+SUM(G13:G15)</f>
-        <v/>
-      </c>
-      <c r="H17" s="5">
-        <f>H2+H5+H6+H7+H10+H11+H12+SUM(H13:H15)</f>
-        <v/>
-      </c>
-      <c r="I17" s="5">
-        <f>I2+I5+I6+I7+I10+I11+I12+SUM(I13:I15)</f>
-        <v/>
-      </c>
-      <c r="J17" s="5">
-        <f>SUM(D17:I17)</f>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3">
+        <f>IF(C17="R$",SUM(D17:I17),"")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>MÍDIA</t>
+          <t>CUSTO OPERACIONAL (sem mídia)</t>
         </is>
       </c>
       <c r="D18" s="5">
-        <f>D9</f>
+        <f>D2+D5+D6+D7+D8+D11+D12+D13+SUM(D14:D16)</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>E9</f>
+        <f>E2+E5+E6+E7+E8+E11+E12+E13+SUM(E14:E16)</f>
         <v/>
       </c>
       <c r="F18" s="5">
-        <f>F9</f>
+        <f>F2+F5+F6+F7+F8+F11+F12+F13+SUM(F14:F16)</f>
         <v/>
       </c>
       <c r="G18" s="5">
-        <f>G9</f>
+        <f>G2+G5+G6+G7+G8+G11+G12+G13+SUM(G14:G16)</f>
         <v/>
       </c>
       <c r="H18" s="5">
-        <f>H9</f>
+        <f>H2+H5+H6+H7+H8+H11+H12+H13+SUM(H14:H16)</f>
         <v/>
       </c>
       <c r="I18" s="5">
-        <f>I9</f>
+        <f>I2+I5+I6+I7+I8+I11+I12+I13+SUM(I14:I16)</f>
         <v/>
       </c>
       <c r="J18" s="5">
@@ -2008,35 +2021,70 @@
     <row r="19">
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>CUSTO FIXO TOTAL DO MÊS</t>
+          <t>MÍDIA</t>
         </is>
       </c>
       <c r="D19" s="5">
-        <f>D17+D18</f>
+        <f>D10</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>E17+E18</f>
+        <f>E10</f>
         <v/>
       </c>
       <c r="F19" s="5">
-        <f>F17+F18</f>
+        <f>F10</f>
         <v/>
       </c>
       <c r="G19" s="5">
-        <f>G17+G18</f>
+        <f>G10</f>
         <v/>
       </c>
       <c r="H19" s="5">
-        <f>H17+H18</f>
+        <f>H10</f>
         <v/>
       </c>
       <c r="I19" s="5">
-        <f>I17+I18</f>
+        <f>I10</f>
         <v/>
       </c>
       <c r="J19" s="5">
         <f>SUM(D19:I19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>CUSTO FIXO TOTAL DO MÊS</t>
+        </is>
+      </c>
+      <c r="D20" s="5">
+        <f>D18+D19</f>
+        <v/>
+      </c>
+      <c r="E20" s="5">
+        <f>E18+E19</f>
+        <v/>
+      </c>
+      <c r="F20" s="5">
+        <f>F18+F19</f>
+        <v/>
+      </c>
+      <c r="G20" s="5">
+        <f>G18+G19</f>
+        <v/>
+      </c>
+      <c r="H20" s="5">
+        <f>H18+H19</f>
+        <v/>
+      </c>
+      <c r="I20" s="5">
+        <f>I18+I19</f>
+        <v/>
+      </c>
+      <c r="J20" s="5">
+        <f>SUM(D20:I20)</f>
         <v/>
       </c>
     </row>

</xml_diff>